<commit_message>
feat: actualizar formulas del simulador fiscal segun excel
</commit_message>
<xml_diff>
--- a/CursosIEDCH/public/CALCULADORA FISCAL SIAI.xlsx
+++ b/CursosIEDCH/public/CALCULADORA FISCAL SIAI.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ventas 1\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sergi\.gemini\antigravity\scratch\CursosIEDCH\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC72B2E3-487A-49BC-A085-8430A92FD0F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{09DDA787-A620-4656-B32C-84F4BB131F4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4785" yWindow="3435" windowWidth="11415" windowHeight="15375" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="592" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Simulador" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>SIMULADOR DE RETENCIONES Y PAGOS</t>
   </si>
@@ -35,10 +48,6 @@
   </si>
   <si>
     <t>CONCEPTOS / RUBROS</t>
-  </si>
-  <si>
-    <t>RESICO (P.
-FÍSICA)</t>
   </si>
   <si>
     <t>ACTIVIDAD
@@ -87,6 +96,12 @@
   </si>
   <si>
     <t>Pago Neto a Depositar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RESICO </t>
+  </si>
+  <si>
+    <t>&lt;&lt;</t>
   </si>
 </sst>
 </file>
@@ -96,7 +111,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="\$#,##0.00;\(\$#,##0.00\);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -109,27 +124,39 @@
       <sz val="16"/>
       <color rgb="FF1F4E78"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF1F4E78"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -200,7 +227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -234,6 +261,7 @@
     <xf numFmtId="164" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -536,8 +564,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
+  <dimension ref="A1:E29"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" outlineLevelRow="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="4" width="18" customWidth="1"/>
@@ -549,17 +580,27 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3" s="13">
+        <v>1000</v>
+      </c>
+    </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="B4" s="13">
+        <f>B3*0.16</f>
+        <v>160</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="3">
-        <v>1000</v>
+        <f>B3+B4</f>
+        <v>1160</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -575,63 +616,63 @@
         <v>4</v>
       </c>
       <c r="B9" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="D9" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>7</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="8">
         <f>$B$5*$B$6</f>
-        <v>20000</v>
+        <v>23200</v>
       </c>
       <c r="C10" s="8">
         <f>$B$5*$B$6</f>
-        <v>20000</v>
+        <v>23200</v>
       </c>
       <c r="D10" s="8">
         <f>$B$5*$B$6</f>
-        <v>20000</v>
+        <v>23200</v>
       </c>
       <c r="E10" s="8">
         <f>$B$5*$B$6</f>
-        <v>20000</v>
+        <v>23200</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="10">
         <f>B10*0.036*1.16</f>
-        <v>835.19999999999993</v>
+        <v>968.83199999999988</v>
       </c>
       <c r="C11" s="10">
         <f>C10*0.036*1.16</f>
-        <v>835.19999999999993</v>
+        <v>968.83199999999988</v>
       </c>
       <c r="D11" s="10">
         <f>D10*0.036*1.16</f>
-        <v>835.19999999999993</v>
+        <v>968.83199999999988</v>
       </c>
       <c r="E11" s="10">
         <f>E10*0.036*1.16</f>
-        <v>835.19999999999993</v>
+        <v>968.83199999999988</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" s="10">
         <f>$B$6*3*1.16</f>
@@ -650,80 +691,80 @@
         <v>69.599999999999994</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" s="8">
         <f>B10-B11-B12</f>
-        <v>19095.2</v>
+        <v>22161.568000000003</v>
       </c>
       <c r="C13" s="8">
         <f>C10-C11-C12</f>
-        <v>19095.2</v>
+        <v>22161.568000000003</v>
       </c>
       <c r="D13" s="8">
         <f>D10-D11-D12</f>
-        <v>19095.2</v>
+        <v>22161.568000000003</v>
       </c>
       <c r="E13" s="8">
         <f>E10-E11-E12</f>
-        <v>19095.2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+        <v>22161.568000000003</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" s="8">
         <f>B13*0.5</f>
-        <v>9547.6</v>
+        <v>11080.784000000001</v>
       </c>
       <c r="C14" s="8">
         <f>C13*0.5</f>
-        <v>9547.6</v>
+        <v>11080.784000000001</v>
       </c>
       <c r="D14" s="8">
         <f>D13*0.5</f>
-        <v>9547.6</v>
+        <v>11080.784000000001</v>
       </c>
       <c r="E14" s="8">
         <f>E13*0.5</f>
-        <v>9547.6</v>
+        <v>11080.784000000001</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" s="8">
         <f>B14/1.16</f>
-        <v>8230.6896551724149</v>
+        <v>9552.4000000000015</v>
       </c>
       <c r="C15" s="8">
         <f>C14/1.16</f>
-        <v>8230.6896551724149</v>
+        <v>9552.4000000000015</v>
       </c>
       <c r="D15" s="8">
         <f>D14</f>
-        <v>9547.6</v>
+        <v>11080.784000000001</v>
       </c>
       <c r="E15" s="8">
         <f>E14/1.16</f>
-        <v>8230.6896551724149</v>
+        <v>9552.4000000000015</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" s="10">
         <f>B15*0.16</f>
-        <v>1316.9103448275864</v>
+        <v>1528.3840000000002</v>
       </c>
       <c r="C16" s="10">
         <f>C15*0.16</f>
-        <v>1316.9103448275864</v>
+        <v>1528.3840000000002</v>
       </c>
       <c r="D16" s="10">
         <f>0</f>
@@ -731,45 +772,45 @@
       </c>
       <c r="E16" s="10">
         <f>E15*0.16</f>
-        <v>1316.9103448275864</v>
+        <v>1528.3840000000002</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" s="8">
         <f>B15+B16</f>
-        <v>9547.6000000000022</v>
+        <v>11080.784000000001</v>
       </c>
       <c r="C17" s="8">
         <f>C15+C16</f>
-        <v>9547.6000000000022</v>
+        <v>11080.784000000001</v>
       </c>
       <c r="D17" s="8">
         <f>D15+D16</f>
-        <v>9547.6</v>
+        <v>11080.784000000001</v>
       </c>
       <c r="E17" s="8">
         <f>E15+E16</f>
-        <v>9547.6000000000022</v>
+        <v>11080.784000000001</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" s="10">
         <f>B15*0.0125</f>
-        <v>102.88362068965519</v>
+        <v>119.40500000000003</v>
       </c>
       <c r="C18" s="10">
         <f>C15*0.1</f>
-        <v>823.06896551724151</v>
+        <v>955.24000000000024</v>
       </c>
       <c r="D18" s="10">
         <f>D15*0.0615</f>
-        <v>587.17740000000003</v>
+        <v>681.4682160000001</v>
       </c>
       <c r="E18" s="10">
         <f>0</f>
@@ -778,15 +819,15 @@
     </row>
     <row r="19" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B19" s="10">
-        <f>0</f>
-        <v>0</v>
+        <f>B15*10.6667%</f>
+        <v>1018.9258508000003</v>
       </c>
       <c r="C19" s="10">
-        <f>0</f>
-        <v>0</v>
+        <f>C15*10.6667%</f>
+        <v>1018.9258508000003</v>
       </c>
       <c r="D19" s="10">
         <f>0</f>
@@ -799,19 +840,19 @@
     </row>
     <row r="20" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" s="10">
         <f>SUM(B18:B19)</f>
-        <v>102.88362068965519</v>
+        <v>1138.3308508000002</v>
       </c>
       <c r="C20" s="10">
         <f>SUM(C18:C19)</f>
-        <v>823.06896551724151</v>
+        <v>1974.1658508000005</v>
       </c>
       <c r="D20" s="10">
         <f>SUM(D18:D19)</f>
-        <v>587.17740000000003</v>
+        <v>681.4682160000001</v>
       </c>
       <c r="E20" s="10">
         <f>SUM(E18:E19)</f>
@@ -820,23 +861,28 @@
     </row>
     <row r="21" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" s="12">
         <f>B17-B20</f>
-        <v>9444.7163793103464</v>
+        <v>9942.4531492000006</v>
       </c>
       <c r="C21" s="12">
         <f>C17-C20</f>
-        <v>8724.5310344827612</v>
+        <v>9106.6181492000014</v>
       </c>
       <c r="D21" s="12">
         <f>D17-D20</f>
-        <v>8960.4225999999999</v>
+        <v>10399.315784000002</v>
       </c>
       <c r="E21" s="12">
         <f>E17-E20</f>
-        <v>9547.6000000000022</v>
+        <v>11080.784000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D29" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>